<commit_message>
Update test, group label warning was removed
</commit_message>
<xml_diff>
--- a/test/pyxform-warning.xlsx
+++ b/test/pyxform-warning.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="28908"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10224"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yanokwa/Documents/Work/Nafundi/Code/nafundi/xlsform-offline/test/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ln/Documents/projects/odk/pyxform-http/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48EBFFA0-AAC6-084D-8EC3-02B5F4D30188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3500" yWindow="6100" windowWidth="25520" windowHeight="13940" tabRatio="500"/>
+    <workbookView xWindow="3500" yWindow="6100" windowWidth="25520" windowHeight="13940" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -20,10 +21,21 @@
     <definedName name="OLE_LINK38" localSheetId="0">survey!#REF!</definedName>
     <definedName name="OLE_LINK51" localSheetId="0">survey!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="130407" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -56,19 +68,19 @@
     <t>what is your name</t>
   </si>
   <si>
-    <t>begin group</t>
+    <t>begin repeat</t>
   </si>
   <si>
-    <t>end group</t>
+    <t>repeat</t>
   </si>
   <si>
-    <t>group</t>
+    <t>end repeat</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -324,10 +336,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="191">
@@ -528,6 +539,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -854,7 +868,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -874,42 +888,42 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upgrade to pyxform 4.3.0 (#62)
</commit_message>
<xml_diff>
--- a/test/pyxform-warning.xlsx
+++ b/test/pyxform-warning.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="28908"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10224"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yanokwa/Documents/Work/Nafundi/Code/nafundi/xlsform-offline/test/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ln/Documents/projects/odk/pyxform-http/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48EBFFA0-AAC6-084D-8EC3-02B5F4D30188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3500" yWindow="6100" windowWidth="25520" windowHeight="13940" tabRatio="500"/>
+    <workbookView xWindow="3500" yWindow="6100" windowWidth="25520" windowHeight="13940" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -20,10 +21,21 @@
     <definedName name="OLE_LINK38" localSheetId="0">survey!#REF!</definedName>
     <definedName name="OLE_LINK51" localSheetId="0">survey!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="130407" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
@@ -56,19 +68,19 @@
     <t>what is your name</t>
   </si>
   <si>
-    <t>begin group</t>
+    <t>begin repeat</t>
   </si>
   <si>
-    <t>end group</t>
+    <t>repeat</t>
   </si>
   <si>
-    <t>group</t>
+    <t>end repeat</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -324,10 +336,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="191">
@@ -528,6 +539,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -854,7 +868,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -874,42 +888,42 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>